<commit_message>
Regenerate examples and demo GIF under the new name; drop pre-PyPI install note; absolute GIF URL for PyPI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sample_matrix_answered.xlsx
+++ b/examples/sample_matrix_answered.xlsx
@@ -3028,7 +3028,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>baa6d00069283c6d1e3bf44da596c9d0c2a08c325d2ae64e1f93d3cf2234ed1a</t>
+          <t>810505ce6ee48f7ab56a3d39554c3b7bf49599e8372706486d30a420c14dbf2d</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>amagi-shall 0.1.0</t>
+          <t>amagi-federal-compliance-matrix 0.1.0</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>

</xml_diff>